<commit_message>
Realización del event storming de la entidad residente dentro de reservas
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Event Storming/Reservas - Event Storming.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Event Storming/Reservas - Event Storming.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josez\Documents\Universidad IngeSistemas\Diseño Orientado a Objetos(DOO)\VictusProyect\victus-doc\Doo-Doc\Nueva Version Victus\Event Storming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC7A2AE-0325-4C03-B3E7-2059DACF6BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D803920-339C-4590-A210-7EC24C4FCDCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{36012E7C-B3F4-482B-AC16-7CCB81B9AE88}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{36012E7C-B3F4-482B-AC16-7CCB81B9AE88}"/>
   </bookViews>
   <sheets>
     <sheet name="Flujo de eventos en el tiempo" sheetId="61" r:id="rId1"/>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="153">
   <si>
     <t>Descripción</t>
   </si>
@@ -230,9 +230,6 @@
     <t>Acción de eliminar un turno</t>
   </si>
   <si>
-    <t>Información conjunto residencial</t>
-  </si>
-  <si>
     <t>Crear reserva</t>
   </si>
   <si>
@@ -287,45 +284,21 @@
     <t>Eliminar reserva</t>
   </si>
   <si>
-    <t>Información del conjunto residencial al cual se va a registrar un administrador</t>
-  </si>
-  <si>
     <t>Resid-Pol0001</t>
   </si>
   <si>
     <t>Asegurar que los datos requeridos para registrar la información del nuevo residente sean válidos a nivel de tipo de dato,formato, rango, longitud y obligatoriedad.</t>
   </si>
   <si>
-    <t>Modificar administrador</t>
-  </si>
-  <si>
-    <t>Información del conjunto residencial al cual se va a modificar un administrador</t>
-  </si>
-  <si>
     <t>Resid-Pol0002</t>
   </si>
   <si>
-    <t>Se debe asegurar que no exista otro Residente registrado con el mismo tipo y numero de documento de identidad.</t>
-  </si>
-  <si>
-    <t>Información del conjunto residencial al cual se va a buscar un administrador</t>
-  </si>
-  <si>
     <t>Resid-Pol0003</t>
   </si>
   <si>
-    <t>Se debe asegurar que no exista otro Residente registrado con el mismo numero de contacto.</t>
-  </si>
-  <si>
-    <t>Asegurar que el identificador del residente que se desea registrar  no ha haya sido asignado previamente a otro conjunto residencial.</t>
-  </si>
-  <si>
     <t>Resid-Pol0004</t>
   </si>
   <si>
-    <t>Se debe asegurar que no exista otro residente registrado con el mismo correo electronico.</t>
-  </si>
-  <si>
     <t>Registrar turno</t>
   </si>
   <si>
@@ -462,13 +435,287 @@
   </si>
   <si>
     <t>Reservar turno.</t>
+  </si>
+  <si>
+    <t>RegistrarResidente</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La combinación de </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>tipoDocumento</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>numeroDocumento</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>numeroContacto</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>inmueble</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe ser única.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>fechaNacimiento</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe indicar mayoría de edad (si aplica la política).</t>
+    </r>
+  </si>
+  <si>
+    <t>El Residente debe existir.</t>
+  </si>
+  <si>
+    <t>Si se cambian atributos como tipoDocumento, numeroDocumento, numeroContacto o inmueble, la combinación debe seguir siendo única.</t>
+  </si>
+  <si>
+    <t>Modificar Residente</t>
+  </si>
+  <si>
+    <t>Información Residentes</t>
+  </si>
+  <si>
+    <t>Resid-Pol0005</t>
+  </si>
+  <si>
+    <t>Resid-Pol0006</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Residente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe existir.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verificar que no haya dependencias en otros sistemas o contextos (como reservas de zonas comunes) antes de eliminar al residente.</t>
+  </si>
+  <si>
+    <t>Residente registrado</t>
+  </si>
+  <si>
+    <t>Actualizar datos de contacto</t>
+  </si>
+  <si>
+    <t>información del residente de un conjunto residencial.</t>
+  </si>
+  <si>
+    <t>Resid-Pol0007</t>
+  </si>
+  <si>
+    <t>Resid-Pol0008</t>
+  </si>
+  <si>
+    <t>Resid-Pol0009</t>
+  </si>
+  <si>
+    <t>Resid-Pol0011</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Residente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe estar autenticado.</t>
+    </r>
+  </si>
+  <si>
+    <t>El numeroContacto y correoElectronico deben ser válidos y únicos dentro del contexto.</t>
+  </si>
+  <si>
+    <t>Datos actualizados</t>
+  </si>
+  <si>
+    <t>Actualizar datos de contacto.</t>
+  </si>
+  <si>
+    <t>Cambiar Contrasena</t>
+  </si>
+  <si>
+    <t>Acción de actualizar la contraseña de un residente de un conjunto residencial</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Residente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> debe estar autenticado y la </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>contraseña</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> actual debe ser correcta.</t>
+    </r>
+  </si>
+  <si>
+    <t>La nueva contraseña debe cumplir con las políticas de seguridad establecidas.</t>
+  </si>
+  <si>
+    <t>Contraseña actualizada</t>
+  </si>
+  <si>
+    <t>Cambiar contraseña</t>
+  </si>
+  <si>
+    <t>Buscar Residente</t>
+  </si>
+  <si>
+    <t>Acción de buscar un residente de un conjunto residencial</t>
+  </si>
+  <si>
+    <t>Resid-Pol00010</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> El Residente debe existir.</t>
+  </si>
+  <si>
+    <t>Residente Buscado</t>
+  </si>
+  <si>
+    <t>Eliminar Residente</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -526,8 +773,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="25">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -654,8 +906,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -847,19 +1117,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -871,33 +1128,13 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -907,7 +1144,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -986,13 +1223,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1000,27 +1231,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1042,20 +1297,123 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1066,79 +1424,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1148,104 +1439,123 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1678,21 +1988,21 @@
       <c r="A1" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="39"/>
-      <c r="D1" s="40"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="41" t="s">
-        <v>97</v>
-      </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="42"/>
+      <c r="B2" s="47" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="47"/>
+      <c r="D2" s="48"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
@@ -1713,12 +2023,12 @@
         <v>33</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="43" t="str">
+      <c r="D4" s="49" t="str">
         <f>$B$1</f>
         <v>Reservas</v>
       </c>
@@ -1728,24 +2038,24 @@
         <v>31</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="44"/>
+      <c r="D5" s="50"/>
     </row>
     <row r="6" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
         <v>32</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="45"/>
+      <c r="D6" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1791,84 +2101,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57" t="str">
+      <c r="B2" s="62" t="str">
         <f>'Listado Objetos de Dominio'!A5</f>
         <v>Turno</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="59" t="str">
+      <c r="B3" s="64" t="str">
         <f>'Listado Objetos de Dominio'!B5</f>
         <v>Objeto de dominio que representa uno de los turnos que representan un bloque de tiempo que el residente podrá reservar.</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="60"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="66"/>
       <c r="D4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="E4" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="61"/>
-      <c r="G4" s="62" t="s">
+      <c r="F4" s="67"/>
+      <c r="G4" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="68"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -1878,52 +2188,52 @@
       <c r="K4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="63" t="s">
+      <c r="L4" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="64" t="s">
+      <c r="M4" s="70" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="61"/>
-      <c r="G5" s="65" t="s">
+      <c r="F5" s="67"/>
+      <c r="G5" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="65"/>
-      <c r="I5" s="67" t="s">
+      <c r="H5" s="71"/>
+      <c r="I5" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="68" t="s">
+      <c r="J5" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="66" t="s">
+      <c r="K5" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="63"/>
-      <c r="M5" s="64"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="70"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="71"/>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="70"/>
+      <c r="A6" s="77"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="76"/>
       <c r="E6" s="12" t="s">
         <v>21</v>
       </c>
@@ -1936,391 +2246,395 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="66"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="64"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="70"/>
     </row>
     <row r="7" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="85" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="85" t="s">
+      <c r="B7" s="79" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="101" t="s">
+      <c r="D7" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="101" t="s">
+      <c r="E7" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="101" t="s">
+      <c r="F7" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="99" t="s">
+      <c r="G7" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="99" t="s">
+      <c r="H7" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="I7" s="79"/>
+      <c r="J7" s="79" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="79"/>
+      <c r="L7" s="79" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" s="33" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="78"/>
+      <c r="B8" s="79"/>
+      <c r="C8" s="79"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="80" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="80" t="s">
+        <v>90</v>
+      </c>
+      <c r="I8" s="79"/>
+      <c r="J8" s="79"/>
+      <c r="K8" s="79"/>
+      <c r="L8" s="79"/>
+      <c r="M8" s="79" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="78"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="81"/>
+      <c r="H9" s="81"/>
+      <c r="I9" s="79"/>
+      <c r="J9" s="79"/>
+      <c r="K9" s="79"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+    </row>
+    <row r="10" spans="1:14" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="78" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="88" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="88" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="52"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52"/>
+      <c r="G10" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88" t="s">
+        <v>48</v>
+      </c>
+      <c r="K10" s="89"/>
+      <c r="L10" s="88" t="s">
+        <v>34</v>
+      </c>
+      <c r="M10" s="88" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="78"/>
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="82" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="84" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="84"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88"/>
+    </row>
+    <row r="12" spans="1:14" ht="94.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="78"/>
+      <c r="B12" s="88"/>
+      <c r="C12" s="88"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="85"/>
+      <c r="I12" s="88"/>
+      <c r="J12" s="88"/>
+      <c r="K12" s="85"/>
+      <c r="L12" s="88"/>
+      <c r="M12" s="88"/>
+    </row>
+    <row r="13" spans="1:14" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="52"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="H13" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="59"/>
+      <c r="J13" s="59" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" s="59"/>
+      <c r="L13" s="59" t="s">
+        <v>34</v>
+      </c>
+      <c r="M13" s="59" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="54"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85" t="s">
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="60"/>
+      <c r="L14" s="60"/>
+      <c r="M14" s="60"/>
+    </row>
+    <row r="15" spans="1:14" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="86" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="86" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="86" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="86" t="s">
+        <v>99</v>
+      </c>
+      <c r="I15" s="86"/>
+      <c r="J15" s="86" t="s">
+        <v>77</v>
+      </c>
+      <c r="K15" s="86"/>
+      <c r="L15" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="K7" s="85"/>
-      <c r="L7" s="85" t="s">
+      <c r="M15" s="40" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="54"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="52"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="87"/>
+      <c r="J16" s="87"/>
+      <c r="K16" s="87"/>
+      <c r="L16" s="87"/>
+      <c r="M16" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="M7" s="86" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="46"/>
-      <c r="B8" s="85"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="F8" s="101"/>
-      <c r="G8" s="87" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8" s="87" t="s">
-        <v>99</v>
-      </c>
-      <c r="I8" s="85"/>
-      <c r="J8" s="85"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="85"/>
-      <c r="M8" s="85" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="46"/>
-      <c r="B9" s="85"/>
-      <c r="C9" s="85"/>
-      <c r="D9" s="101"/>
-      <c r="E9" s="101"/>
-      <c r="F9" s="101"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="85"/>
-      <c r="J9" s="85"/>
-      <c r="K9" s="85"/>
-      <c r="L9" s="85"/>
-      <c r="M9" s="85"/>
-    </row>
-    <row r="10" spans="1:14" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="46" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="89" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="89" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="101"/>
-      <c r="E10" s="101"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="102" t="s">
-        <v>100</v>
-      </c>
-      <c r="H10" s="100" t="s">
+    </row>
+    <row r="17" spans="1:13" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="53" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="I10" s="89"/>
-      <c r="J10" s="89" t="s">
-        <v>48</v>
-      </c>
-      <c r="K10" s="91"/>
-      <c r="L10" s="89" t="s">
+      <c r="C17" s="57" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" s="52"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="52"/>
+      <c r="G17" s="42" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" s="57"/>
+      <c r="J17" s="57" t="s">
+        <v>109</v>
+      </c>
+      <c r="K17" s="57"/>
+      <c r="L17" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="M10" s="89" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="46"/>
-      <c r="B11" s="89"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="101"/>
-      <c r="E11" s="101"/>
-      <c r="F11" s="101"/>
-      <c r="G11" s="90" t="s">
+      <c r="M17" s="57" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="54"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="42" t="s">
+        <v>105</v>
+      </c>
+      <c r="H18" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="I18" s="58"/>
+      <c r="J18" s="58"/>
+      <c r="K18" s="58"/>
+      <c r="L18" s="58"/>
+      <c r="M18" s="58"/>
+    </row>
+    <row r="19" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="53" t="s">
         <v>101</v>
       </c>
-      <c r="H11" s="92" t="s">
-        <v>103</v>
-      </c>
-      <c r="I11" s="89"/>
-      <c r="J11" s="89"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="89"/>
-      <c r="M11" s="89"/>
-    </row>
-    <row r="12" spans="1:14" ht="94.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="46"/>
-      <c r="B12" s="89"/>
-      <c r="C12" s="89"/>
-      <c r="D12" s="101"/>
-      <c r="E12" s="101"/>
-      <c r="F12" s="101"/>
-      <c r="G12" s="93"/>
-      <c r="H12" s="94"/>
-      <c r="I12" s="89"/>
-      <c r="J12" s="89"/>
-      <c r="K12" s="94"/>
-      <c r="L12" s="89"/>
-      <c r="M12" s="89"/>
-    </row>
-    <row r="13" spans="1:14" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="104" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="104" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="101"/>
-      <c r="E13" s="101"/>
-      <c r="F13" s="101"/>
-      <c r="G13" s="95" t="s">
-        <v>105</v>
-      </c>
-      <c r="H13" s="95" t="s">
-        <v>102</v>
-      </c>
-      <c r="I13" s="104"/>
-      <c r="J13" s="104" t="s">
-        <v>83</v>
-      </c>
-      <c r="K13" s="104"/>
-      <c r="L13" s="104" t="s">
-        <v>34</v>
-      </c>
-      <c r="M13" s="104" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="48"/>
-      <c r="B14" s="105"/>
-      <c r="C14" s="105"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="101"/>
-      <c r="F14" s="101"/>
-      <c r="G14" s="95" t="s">
-        <v>106</v>
-      </c>
-      <c r="H14" s="103" t="s">
+      <c r="B19" s="55" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="52"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="105"/>
-      <c r="L14" s="105"/>
-      <c r="M14" s="105"/>
-    </row>
-    <row r="15" spans="1:14" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="47" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="96" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="96" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="101"/>
-      <c r="E15" s="101"/>
-      <c r="F15" s="101"/>
-      <c r="G15" s="96" t="s">
-        <v>109</v>
-      </c>
-      <c r="H15" s="96" t="s">
-        <v>108</v>
-      </c>
-      <c r="I15" s="96"/>
-      <c r="J15" s="96" t="s">
-        <v>86</v>
-      </c>
-      <c r="K15" s="96"/>
-      <c r="L15" s="96" t="s">
-        <v>34</v>
-      </c>
-      <c r="M15" s="106" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="48"/>
-      <c r="B16" s="97"/>
-      <c r="C16" s="97"/>
-      <c r="D16" s="101"/>
-      <c r="E16" s="101"/>
-      <c r="F16" s="101"/>
-      <c r="G16" s="97"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="97"/>
-      <c r="J16" s="97"/>
-      <c r="K16" s="97"/>
-      <c r="L16" s="97"/>
-      <c r="M16" s="98" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="B17" s="108" t="s">
+      <c r="H19" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="I19" s="55"/>
+      <c r="J19" s="55" t="s">
+        <v>116</v>
+      </c>
+      <c r="K19" s="55"/>
+      <c r="L19" s="55" t="s">
+        <v>117</v>
+      </c>
+      <c r="M19" s="55" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="54"/>
+      <c r="B20" s="56"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="108" t="s">
-        <v>112</v>
-      </c>
-      <c r="D17" s="101"/>
-      <c r="E17" s="101"/>
-      <c r="F17" s="101"/>
-      <c r="G17" s="110" t="s">
-        <v>113</v>
-      </c>
-      <c r="H17" s="107" t="s">
+      <c r="H20" s="44" t="s">
         <v>115</v>
       </c>
-      <c r="I17" s="108"/>
-      <c r="J17" s="108" t="s">
-        <v>118</v>
-      </c>
-      <c r="K17" s="108"/>
-      <c r="L17" s="108" t="s">
-        <v>34</v>
-      </c>
-      <c r="M17" s="108" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="48"/>
-      <c r="B18" s="109"/>
-      <c r="C18" s="109"/>
-      <c r="D18" s="101"/>
-      <c r="E18" s="101"/>
-      <c r="F18" s="101"/>
-      <c r="G18" s="110" t="s">
-        <v>114</v>
-      </c>
-      <c r="H18" s="107" t="s">
-        <v>117</v>
-      </c>
-      <c r="I18" s="109"/>
-      <c r="J18" s="109"/>
-      <c r="K18" s="109"/>
-      <c r="L18" s="109"/>
-      <c r="M18" s="109"/>
-    </row>
-    <row r="19" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="B19" s="111" t="s">
-        <v>121</v>
-      </c>
-      <c r="C19" s="111" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" s="101"/>
-      <c r="E19" s="101"/>
-      <c r="F19" s="101"/>
-      <c r="G19" s="113" t="s">
-        <v>116</v>
-      </c>
-      <c r="H19" s="114" t="s">
-        <v>123</v>
-      </c>
-      <c r="I19" s="111"/>
-      <c r="J19" s="111" t="s">
-        <v>125</v>
-      </c>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111" t="s">
-        <v>126</v>
-      </c>
-      <c r="M19" s="111" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="48"/>
-      <c r="B20" s="112"/>
-      <c r="C20" s="112"/>
-      <c r="D20" s="101"/>
-      <c r="E20" s="101"/>
-      <c r="F20" s="101"/>
-      <c r="G20" s="113" t="s">
-        <v>120</v>
-      </c>
-      <c r="H20" s="114" t="s">
-        <v>124</v>
-      </c>
-      <c r="I20" s="112"/>
-      <c r="J20" s="112"/>
-      <c r="K20" s="112"/>
-      <c r="L20" s="112"/>
-      <c r="M20" s="112"/>
+      <c r="I20" s="56"/>
+      <c r="J20" s="56"/>
+      <c r="K20" s="56"/>
+      <c r="L20" s="56"/>
+      <c r="M20" s="56"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H22" s="30"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H23" s="30"/>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H24" s="30"/>
+      <c r="H24" s="28"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H25" s="30"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H26" s="30"/>
+      <c r="H26" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="73">
-    <mergeCell ref="D7:D20"/>
-    <mergeCell ref="E7:E20"/>
-    <mergeCell ref="F7:F20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="M13:M14"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="J10:J12"/>
+    <mergeCell ref="K10:K12"/>
+    <mergeCell ref="L10:L12"/>
+    <mergeCell ref="M10:M12"/>
+    <mergeCell ref="L7:L9"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="G8:G9"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B3:M3"/>
@@ -2337,37 +2651,33 @@
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="J10:J12"/>
-    <mergeCell ref="K10:K12"/>
-    <mergeCell ref="L10:L12"/>
-    <mergeCell ref="M10:M12"/>
-    <mergeCell ref="L7:L9"/>
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="M13:M14"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
     <mergeCell ref="L15:L16"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="D7:D20"/>
+    <mergeCell ref="E7:E20"/>
+    <mergeCell ref="F7:F20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -2381,7 +2691,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3D88CD-1BA6-4157-9522-8201A0FEDE3C}">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -2391,9 +2701,9 @@
     <col min="5" max="6" width="18.88671875" style="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="31.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.21875" style="1" customWidth="1"/>
     <col min="10" max="10" width="43.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.33203125" style="1" customWidth="1"/>
     <col min="12" max="12" width="38" style="1" customWidth="1"/>
     <col min="13" max="13" width="46.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -2406,84 +2716,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57" t="str">
+      <c r="B2" s="62" t="str">
         <f>'Listado Objetos de Dominio'!A6</f>
         <v>Residente</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="59" t="str">
+      <c r="B3" s="64" t="str">
         <f>'Listado Objetos de Dominio'!B6</f>
         <v>Objeto de dominio que representa a un residente que vive dentro de un inmueble en un conjunto residencial</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="60"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="66"/>
       <c r="D4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="E4" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="61"/>
-      <c r="G4" s="62" t="s">
+      <c r="F4" s="67"/>
+      <c r="G4" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="68"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -2493,52 +2803,52 @@
       <c r="K4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="63" t="s">
+      <c r="L4" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="64" t="s">
+      <c r="M4" s="70" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="61"/>
-      <c r="G5" s="65" t="s">
+      <c r="F5" s="67"/>
+      <c r="G5" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="65"/>
-      <c r="I5" s="67" t="s">
+      <c r="H5" s="71"/>
+      <c r="I5" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="68" t="s">
+      <c r="J5" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="66" t="s">
+      <c r="K5" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="63"/>
-      <c r="M5" s="64"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="70"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="71"/>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="70"/>
+      <c r="A6" s="77"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="76"/>
       <c r="E6" s="12" t="s">
         <v>21</v>
       </c>
@@ -2551,238 +2861,419 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="66"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="64"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="72" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="49" t="str">
-        <f>_xlfn.CONCAT("Registrar ",B2)</f>
-        <v>Registrar Residente</v>
-      </c>
-      <c r="C7" s="49" t="str">
+      <c r="I6" s="73"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="70"/>
+    </row>
+    <row r="7" spans="1:14" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="131" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="102" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="102" t="str">
         <f>_xlfn.CONCAT("Acción de registrar un ",B2," para un conjunto residencial.")</f>
         <v>Acción de registrar un Residente para un conjunto residencial.</v>
       </c>
-      <c r="D7" s="49" t="str">
+      <c r="D7" s="131" t="str">
         <f>B2</f>
         <v>Residente</v>
       </c>
-      <c r="E7" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" s="49" t="s">
-        <v>69</v>
-      </c>
-      <c r="G7" s="49" t="s">
-        <v>70</v>
-      </c>
-      <c r="H7" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49" t="str">
+      <c r="E7" s="131" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="131" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" s="103" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="104" t="s">
+        <v>120</v>
+      </c>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102" t="str">
         <f>_xlfn.CONCAT(B2," registrado")</f>
         <v>Residente registrado</v>
       </c>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49" t="str">
+      <c r="K7" s="102"/>
+      <c r="L7" s="102" t="str">
         <f>_xlfn.CONCAT(B2," eliminado")</f>
         <v>Residente eliminado</v>
       </c>
-      <c r="M7" s="33" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="73"/>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="75"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="75"/>
-      <c r="J8" s="75"/>
-      <c r="K8" s="75"/>
-      <c r="L8" s="75"/>
-      <c r="M8" s="33" t="str">
+      <c r="M7" s="105" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="132"/>
+      <c r="B8" s="106"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="132"/>
+      <c r="F8" s="132"/>
+      <c r="G8" s="102" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="127" t="s">
+        <v>121</v>
+      </c>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="106"/>
+      <c r="M8" s="105" t="str">
         <f>_xlfn.CONCAT("Buscar ",B2)</f>
         <v>Buscar Residente</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="74"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="33" t="str">
+      <c r="A9" s="132"/>
+      <c r="B9" s="107"/>
+      <c r="C9" s="107"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="107"/>
+      <c r="H9" s="127"/>
+      <c r="I9" s="107"/>
+      <c r="J9" s="107"/>
+      <c r="K9" s="107"/>
+      <c r="L9" s="107"/>
+      <c r="M9" s="105" t="str">
         <f>_xlfn.CONCAT("Eliminar ",B2)</f>
         <v>Eliminar Residente</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A10" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="27" t="str">
+    <row r="10" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="132"/>
+      <c r="B10" s="129" t="s">
+        <v>147</v>
+      </c>
+      <c r="C10" s="129" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" s="132"/>
+      <c r="E10" s="132"/>
+      <c r="F10" s="132"/>
+      <c r="G10" s="129" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" s="137" t="s">
+        <v>150</v>
+      </c>
+      <c r="I10" s="125"/>
+      <c r="J10" s="129" t="s">
+        <v>151</v>
+      </c>
+      <c r="K10" s="125"/>
+      <c r="L10" s="129" t="s">
+        <v>130</v>
+      </c>
+      <c r="M10" s="126" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="132"/>
+      <c r="B11" s="128"/>
+      <c r="C11" s="128"/>
+      <c r="D11" s="132"/>
+      <c r="E11" s="132"/>
+      <c r="F11" s="132"/>
+      <c r="G11" s="128"/>
+      <c r="H11" s="138"/>
+      <c r="I11" s="125"/>
+      <c r="J11" s="128"/>
+      <c r="K11" s="125"/>
+      <c r="L11" s="128"/>
+      <c r="M11" s="126" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="132"/>
+      <c r="B12" s="130"/>
+      <c r="C12" s="130"/>
+      <c r="D12" s="132"/>
+      <c r="E12" s="132"/>
+      <c r="F12" s="132"/>
+      <c r="G12" s="130"/>
+      <c r="H12" s="139"/>
+      <c r="I12" s="125"/>
+      <c r="J12" s="130"/>
+      <c r="K12" s="125"/>
+      <c r="L12" s="130"/>
+      <c r="M12" s="126" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="132"/>
+      <c r="B13" s="108" t="str">
         <f>_xlfn.CONCAT("Modificar ",B2)</f>
         <v>Modificar Residente</v>
       </c>
-      <c r="C10" s="27" t="str">
+      <c r="C13" s="108" t="str">
         <f>_xlfn.CONCAT("Acción de modificar la información asociada a un ",B2," del conjunto residencial.")</f>
         <v>Acción de modificar la información asociada a un Residente del conjunto residencial.</v>
       </c>
-      <c r="D10" s="27" t="str">
-        <f>B2</f>
-        <v>Residente</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27" t="str">
+      <c r="D13" s="132"/>
+      <c r="E13" s="132"/>
+      <c r="F13" s="132"/>
+      <c r="G13" s="109" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="109" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" s="108"/>
+      <c r="J13" s="108" t="str">
         <f>_xlfn.CONCAT(B2," modificado")</f>
         <v>Residente modificado</v>
       </c>
-      <c r="K10" s="27"/>
-      <c r="L10" s="47" t="str">
+      <c r="K13" s="108"/>
+      <c r="L13" s="108" t="str">
         <f>_xlfn.CONCAT(B2," registrado")</f>
         <v>Residente registrado</v>
       </c>
-      <c r="M10" s="33" t="str">
+      <c r="M13" s="109" t="str">
         <f>_xlfn.CONCAT("Eliminar ",$B$2)</f>
         <v>Eliminar Residente</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="76" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="49" t="str">
-        <f>_xlfn.CONCAT("Buscar ",B2)</f>
-        <v>Buscar Residente</v>
-      </c>
-      <c r="C11" s="49" t="str">
-        <f>_xlfn.CONCAT("Acción de buscar la información asociada a un ",B2," del conjunto residencial.")</f>
-        <v>Acción de buscar la información asociada a un Residente del conjunto residencial.</v>
-      </c>
-      <c r="D11" s="49" t="str">
-        <f>B2</f>
-        <v>Residente</v>
-      </c>
-      <c r="E11" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="49" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" s="49" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" s="49"/>
-      <c r="J11" s="49" t="str">
-        <f>_xlfn.CONCAT(B2," buscado")</f>
-        <v>Residente buscado</v>
-      </c>
-      <c r="K11" s="49"/>
-      <c r="L11" s="54"/>
-      <c r="M11" s="33" t="str">
-        <f>_xlfn.CONCAT("Modificar ",$B$2)</f>
-        <v>Modificar Residente</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="77"/>
-      <c r="B12" s="50"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="50"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="50"/>
-      <c r="G12" s="50"/>
-      <c r="H12" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="I12" s="50"/>
-      <c r="J12" s="50"/>
-      <c r="K12" s="50"/>
-      <c r="L12" s="54"/>
-      <c r="M12" s="34" t="str">
-        <f>_xlfn.CONCAT("Eliminar ",$B$2)</f>
+    <row r="14" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A14" s="132"/>
+      <c r="B14" s="110"/>
+      <c r="C14" s="110"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="132"/>
+      <c r="F14" s="132"/>
+      <c r="G14" s="109" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" s="109" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="110"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="110"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="109" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="132"/>
+      <c r="B15" s="111" t="str">
+        <f>_xlfn.CONCAT("Eliminar ",B2)</f>
         <v>Eliminar Residente</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A13" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="27" t="str">
-        <f>_xlfn.CONCAT("Dar de baja ",B2)</f>
-        <v>Dar de baja Residente</v>
-      </c>
-      <c r="C13" s="27" t="str">
-        <f>_xlfn.CONCAT("Acción de eliminar a un ",B2," de un conjunto residencial.")</f>
-        <v>Acción de eliminar a un Residente de un conjunto residencial.</v>
-      </c>
-      <c r="D13" s="27" t="str">
-        <f>B2</f>
-        <v>Residente</v>
-      </c>
-      <c r="E13" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="H13" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27" t="str">
+      <c r="C15" s="111" t="str">
+        <f>_xlfn.CONCAT("Acción de eliminar la información asociada a un ",B2," del conjunto residencial.")</f>
+        <v>Acción de eliminar la información asociada a un Residente del conjunto residencial.</v>
+      </c>
+      <c r="D15" s="132"/>
+      <c r="E15" s="132"/>
+      <c r="F15" s="132"/>
+      <c r="G15" s="112" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="113" t="s">
+        <v>128</v>
+      </c>
+      <c r="I15" s="111"/>
+      <c r="J15" s="136" t="str">
         <f>_xlfn.CONCAT(B2," eliminado")</f>
         <v>Residente eliminado</v>
       </c>
-      <c r="K13" s="27"/>
-      <c r="L13" s="48"/>
-      <c r="M13" s="33" t="str">
-        <f>_xlfn.CONCAT("Crear ",$B$2)</f>
-        <v>Crear Residente</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="E14" s="35"/>
+      <c r="K15" s="111"/>
+      <c r="L15" s="57" t="s">
+        <v>130</v>
+      </c>
+      <c r="M15" s="134" t="str">
+        <f>_xlfn.CONCAT("Registrar ",$B$2)</f>
+        <v>Registrar Residente</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="133"/>
+      <c r="B16" s="111"/>
+      <c r="C16" s="111"/>
+      <c r="D16" s="132"/>
+      <c r="E16" s="132"/>
+      <c r="F16" s="132"/>
+      <c r="G16" s="112" t="s">
+        <v>133</v>
+      </c>
+      <c r="H16" s="114" t="s">
+        <v>129</v>
+      </c>
+      <c r="I16" s="111"/>
+      <c r="J16" s="136"/>
+      <c r="K16" s="111"/>
+      <c r="L16" s="58"/>
+      <c r="M16" s="135"/>
+    </row>
+    <row r="17" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="131" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="115" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="115" t="str">
+        <f>_xlfn.CONCAT("Acción de actualizar los datos de  ",B2," de un conjunto residencial.")</f>
+        <v>Acción de actualizar los datos de  Residente de un conjunto residencial.</v>
+      </c>
+      <c r="D17" s="132"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="132"/>
+      <c r="G17" s="116" t="s">
+        <v>134</v>
+      </c>
+      <c r="H17" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="I17" s="115"/>
+      <c r="J17" s="115" t="s">
+        <v>139</v>
+      </c>
+      <c r="K17" s="115"/>
+      <c r="L17" s="115" t="s">
+        <v>130</v>
+      </c>
+      <c r="M17" s="119" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="132"/>
+      <c r="B18" s="118"/>
+      <c r="C18" s="118"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="132"/>
+      <c r="G18" s="116" t="s">
+        <v>135</v>
+      </c>
+      <c r="H18" s="116" t="s">
+        <v>138</v>
+      </c>
+      <c r="I18" s="118"/>
+      <c r="J18" s="118"/>
+      <c r="K18" s="118"/>
+      <c r="L18" s="118"/>
+      <c r="M18" s="120" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="132"/>
+      <c r="B19" s="121" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" s="121" t="s">
+        <v>142</v>
+      </c>
+      <c r="D19" s="132"/>
+      <c r="E19" s="132"/>
+      <c r="F19" s="132"/>
+      <c r="G19" s="122" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" s="123" t="s">
+        <v>143</v>
+      </c>
+      <c r="I19" s="121"/>
+      <c r="J19" s="121" t="s">
+        <v>145</v>
+      </c>
+      <c r="K19" s="121"/>
+      <c r="L19" s="121" t="s">
+        <v>130</v>
+      </c>
+      <c r="M19" s="122" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="133"/>
+      <c r="B20" s="124"/>
+      <c r="C20" s="124"/>
+      <c r="D20" s="133"/>
+      <c r="E20" s="133"/>
+      <c r="F20" s="133"/>
+      <c r="G20" s="122" t="s">
+        <v>136</v>
+      </c>
+      <c r="H20" s="122" t="s">
+        <v>144</v>
+      </c>
+      <c r="I20" s="124"/>
+      <c r="J20" s="124"/>
+      <c r="K20" s="124"/>
+      <c r="L20" s="124"/>
+      <c r="M20" s="122" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E21" s="101"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="61">
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="D7:D20"/>
+    <mergeCell ref="E7:E20"/>
+    <mergeCell ref="A7:A16"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="L10:L12"/>
+    <mergeCell ref="J10:J12"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="F7:F20"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="L7:L9"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B3:M3"/>
@@ -2796,34 +3287,8 @@
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="L4:L6"/>
     <mergeCell ref="M4:M6"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="L7:L9"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="L10:L13"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
   </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A1:N1" location="'Listado Objetos de Dominio'!A1" display="&lt;-Volver al inicio" xr:uid="{827E654C-67F5-45D4-9416-536CC2969F91}"/>
   </hyperlinks>
@@ -2859,84 +3324,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57" t="str">
+      <c r="B2" s="62" t="str">
         <f>'Listado Objetos de Dominio'!A4</f>
         <v>Reserva</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="59" t="str">
+      <c r="B3" s="64" t="str">
         <f>'Listado Objetos de Dominio'!B4</f>
         <v>Objeto de dominio que representa a cada una de las reservas creadas por los residente según una zona comun que esta condicionada con una agenda y según la disponibilidad de turno poder reservar el espacio.</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="60"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="55"/>
+      <c r="C4" s="66"/>
       <c r="D4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="E4" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="61"/>
-      <c r="G4" s="62" t="s">
+      <c r="F4" s="67"/>
+      <c r="G4" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="68"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -2946,52 +3411,52 @@
       <c r="K4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="83" t="s">
+      <c r="L4" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="84" t="s">
+      <c r="M4" s="96" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="61"/>
-      <c r="G5" s="65" t="s">
+      <c r="F5" s="67"/>
+      <c r="G5" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="65"/>
-      <c r="I5" s="67" t="s">
+      <c r="H5" s="71"/>
+      <c r="I5" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="68" t="s">
+      <c r="J5" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="66" t="s">
+      <c r="K5" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="83"/>
-      <c r="M5" s="84"/>
+      <c r="L5" s="95"/>
+      <c r="M5" s="96"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="71"/>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="70"/>
+      <c r="A6" s="77"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="76"/>
       <c r="E6" s="12" t="s">
         <v>21</v>
       </c>
@@ -3004,310 +3469,308 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="66"/>
-      <c r="L6" s="83"/>
-      <c r="M6" s="84"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="95"/>
+      <c r="M6" s="96"/>
     </row>
     <row r="7" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="98" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="51" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="47" t="s">
+      <c r="B7" s="92" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="92" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="51" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="47" t="s">
-        <v>53</v>
-      </c>
       <c r="G7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="11"/>
+      <c r="J7" s="92" t="s">
+        <v>82</v>
+      </c>
+      <c r="K7" s="11"/>
+      <c r="L7" s="92" t="s">
+        <v>65</v>
+      </c>
+      <c r="M7" s="32" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="100"/>
+      <c r="B8" s="93"/>
+      <c r="C8" s="91"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="91"/>
+      <c r="G8" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="11"/>
+      <c r="J8" s="93"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="93"/>
+      <c r="M8" s="32" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="100"/>
+      <c r="B9" s="93"/>
+      <c r="C9" s="91"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="93"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="93"/>
+      <c r="M9" s="92" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="100"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="91"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="91"/>
+      <c r="G10" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="51" t="s">
-        <v>91</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="51" t="s">
-        <v>66</v>
-      </c>
-      <c r="M7" s="38" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="82"/>
-      <c r="B8" s="52"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="38" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="82"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="H9" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="51" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="82"/>
-      <c r="B10" s="52"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="52"/>
-      <c r="E10" s="52"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="H10" s="31" t="s">
-        <v>56</v>
-      </c>
       <c r="I10" s="25"/>
-      <c r="J10" s="52"/>
+      <c r="J10" s="93"/>
       <c r="K10" s="25"/>
-      <c r="L10" s="52"/>
-      <c r="M10" s="52"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
     </row>
     <row r="11" spans="1:14" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="81"/>
-      <c r="B11" s="53"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="48"/>
+      <c r="A11" s="99"/>
+      <c r="B11" s="94"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="93"/>
+      <c r="E11" s="94"/>
+      <c r="F11" s="54"/>
       <c r="G11" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>96</v>
+        <v>86</v>
+      </c>
+      <c r="H11" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="I11" s="25"/>
-      <c r="J11" s="53"/>
+      <c r="J11" s="94"/>
       <c r="K11" s="25"/>
-      <c r="L11" s="53"/>
-      <c r="M11" s="53"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="94"/>
     </row>
     <row r="12" spans="1:14" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="51" t="s">
+      <c r="B12" s="92" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="47" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="52"/>
-      <c r="E12" s="51" t="s">
+      <c r="D12" s="93"/>
+      <c r="E12" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="51" t="s">
-        <v>94</v>
-      </c>
-      <c r="H12" s="47" t="s">
-        <v>56</v>
-      </c>
-      <c r="I12" s="51"/>
-      <c r="J12" s="79" t="s">
+      <c r="F12" s="53" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="92" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="53" t="s">
+        <v>55</v>
+      </c>
+      <c r="I12" s="92"/>
+      <c r="J12" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="K12" s="51"/>
-      <c r="L12" s="79" t="s">
+      <c r="K12" s="92"/>
+      <c r="L12" s="97" t="s">
         <v>36</v>
       </c>
-      <c r="M12" s="36" t="s">
-        <v>67</v>
+      <c r="M12" s="30" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="53"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="52"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="53"/>
-      <c r="J13" s="79"/>
-      <c r="K13" s="53"/>
-      <c r="L13" s="79"/>
-      <c r="M13" s="36" t="s">
-        <v>68</v>
+      <c r="B13" s="94"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="93"/>
+      <c r="E13" s="93"/>
+      <c r="F13" s="91"/>
+      <c r="G13" s="93"/>
+      <c r="H13" s="91"/>
+      <c r="I13" s="94"/>
+      <c r="J13" s="97"/>
+      <c r="K13" s="94"/>
+      <c r="L13" s="97"/>
+      <c r="M13" s="30" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="C14" s="47" t="s">
+      <c r="B14" s="53" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="93"/>
+      <c r="E14" s="93"/>
+      <c r="F14" s="91"/>
+      <c r="G14" s="93"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="92"/>
+      <c r="J14" s="92" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" s="92"/>
+      <c r="L14" s="92" t="s">
+        <v>36</v>
+      </c>
+      <c r="M14" s="30" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="91"/>
+      <c r="C15" s="91"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="93"/>
+      <c r="F15" s="91"/>
+      <c r="G15" s="93"/>
+      <c r="H15" s="91"/>
+      <c r="I15" s="93"/>
+      <c r="J15" s="93"/>
+      <c r="K15" s="93"/>
+      <c r="L15" s="93"/>
+      <c r="M15" s="30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="99"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="93"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="91"/>
+      <c r="G16" s="93"/>
+      <c r="H16" s="91"/>
+      <c r="I16" s="94"/>
+      <c r="J16" s="94"/>
+      <c r="K16" s="94"/>
+      <c r="L16" s="94"/>
+      <c r="M16" s="30" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="51"/>
-      <c r="J14" s="51" t="s">
-        <v>93</v>
-      </c>
-      <c r="K14" s="51"/>
-      <c r="L14" s="51" t="s">
+      <c r="C17" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="91"/>
+      <c r="G17" s="93"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="92"/>
+      <c r="J17" s="92" t="s">
+        <v>38</v>
+      </c>
+      <c r="K17" s="92"/>
+      <c r="L17" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="M14" s="36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="80" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="52"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="52"/>
-      <c r="L15" s="52"/>
-      <c r="M15" s="36" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="81"/>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="54"/>
-      <c r="I16" s="53"/>
-      <c r="J16" s="53"/>
-      <c r="K16" s="53"/>
-      <c r="L16" s="53"/>
-      <c r="M16" s="36" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="47" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="47" t="s">
-        <v>65</v>
-      </c>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="52"/>
-      <c r="H17" s="54"/>
-      <c r="I17" s="51"/>
-      <c r="J17" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="K17" s="51"/>
-      <c r="L17" s="51" t="s">
-        <v>36</v>
-      </c>
-      <c r="M17" s="79" t="s">
-        <v>51</v>
+      <c r="M17" s="97" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="53"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="53"/>
-      <c r="K18" s="53"/>
-      <c r="L18" s="53"/>
-      <c r="M18" s="79"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="94"/>
+      <c r="E18" s="94"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="94"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="94"/>
+      <c r="J18" s="94"/>
+      <c r="K18" s="94"/>
+      <c r="L18" s="94"/>
+      <c r="M18" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="L7:L11"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="L4:L6"/>
-    <mergeCell ref="M4:M6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="M9:M11"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="E7:E11"/>
+    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="K14:K16"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="L14:L16"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="B17:B18"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="I12:I13"/>
@@ -3324,22 +3787,24 @@
     <mergeCell ref="E12:E18"/>
     <mergeCell ref="F12:F18"/>
     <mergeCell ref="J7:J11"/>
-    <mergeCell ref="M9:M11"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="F7:F11"/>
-    <mergeCell ref="K14:K16"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="L14:L16"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="M4:M6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="L7:L11"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{804E2C57-E5A8-4901-8BC4-4B63A7C4FA3E}"/>
@@ -3352,6 +3817,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C279D002CEC08F42B7087C30E58D0266" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e5713f579c7011938dc4987ae8981b8f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3219184d-29ab-4105-b29c-8e343e335d59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae0a0ff84a3c6712467f60982d6e378d" ns2:_="">
     <xsd:import namespace="3219184d-29ab-4105-b29c-8e343e335d59"/>
@@ -3495,12 +3966,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3511,6 +3976,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2038022-656B-4A1B-A485-51A1972238BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ff57c5a0-3efd-4333-8513-2b909ca014ae"/>
+    <ds:schemaRef ds:uri="0d2457a1-fe8a-4cb2-a5c3-c59e87d2493e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AEECCE0-61F9-4782-94C5-382F8EFF459D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3528,23 +4010,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2038022-656B-4A1B-A485-51A1972238BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ff57c5a0-3efd-4333-8513-2b909ca014ae"/>
-    <ds:schemaRef ds:uri="0d2457a1-fe8a-4cb2-a5c3-c59e87d2493e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6724C681-8A04-4D66-BB1C-57F7466573C0}">
   <ds:schemaRefs>

</xml_diff>